<commit_message>
Update story-tracker.xlsx and run-log.md with Run #2 data (stories 11-20)
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1023,6 +1023,386 @@
       <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>She blamed teachers. Then watched the footage.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>blamed-teachers-then-watched-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>They merged two great teams. Both collapsed.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>merged-two-great-teams-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>8</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Every test passed. The diesel was dirty.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>vw-clean-diesel-dirty-data-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>He said IBM doesn't need a vision. It needed customers.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>gerstner-ibm-no-vision-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>8</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>They invented the future. Then buried it.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>kodak-invented-future-buried-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Better teams reported more errors. Not fewer.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>edmondson-better-teams-more-errors-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>He put employees first. Customers came second. Profits came anyway.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>kelleher-southwest-employees-first-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>8</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Move fast and break things. They broke everything.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>uber-move-fast-lose-everything-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>8</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Every KPI was green. Every person was leaving.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>every-kpi-green-everyone-leaving-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>8</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>The staff meeting lasted 11 minutes. It saved the school.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>eleven-minute-meeting-saved-school-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>8</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>GitHub</t>
         </is>
       </c>
     </row>
@@ -1081,17 +1461,17 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="D2" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -1102,17 +1482,17 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="D3" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -1123,13 +1503,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -1144,13 +1524,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -1165,17 +1545,17 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1186,17 +1566,17 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1376,6 +1756,30 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>11-20</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>82</v>
+      </c>
+      <c r="F3" t="n">
+        <v>250</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1387,7 +1791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1574,6 +1978,108 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>VW Dieselgate</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Volkswagen programmed 11M diesel cars with defeat devices to cheat emissions tests. EPA discovered in 2015. $30B+ in fines.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>IBM/Gerstner Turnaround</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Lou Gerstner joined IBM 1993, rejected grand vision, focused on customer needs. Transformed IBM from hardware to services.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Kodak/Sasson Digital Camera</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Steve Sasson invented digital camera at Kodak in 1975. Management buried it to protect film business. Kodak filed bankruptcy 2012.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Edmondson Psychological Safety</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Amy Edmondson's research showed better hospital teams reported MORE errors, not fewer. Led to psychological safety concept.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Southwest/Kelleher</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Herb Kelleher built Southwest Airlines on employees-first philosophy. 47 consecutive years of profitability.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Uber/Kalanick</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Travis Kalanick's 'move fast' culture led to scandals, lawsuits, toxic workplace. Forced to resign as CEO in 2017.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update story-tracker.xlsx and run-log.md for Batch 3
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1403,6 +1403,516 @@
       <c r="H21" t="inlineStr">
         <is>
           <t>GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>She fired three coordinators. The role was the problem.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>fired-three-coordinators-same-role</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/fired-three-coordinators-same-role</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>8</v>
+      </c>
+      <c r="J22" t="n">
+        <v>3</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>One question ended the meeting. And started the real one.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>asked-what-are-we-avoiding</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asked-what-are-we-avoiding</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>8</v>
+      </c>
+      <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>The team was working hard. On completely different things.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>mapped-the-workflow-saw-the-gap</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/mapped-the-workflow-saw-the-gap</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>8</v>
+      </c>
+      <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>The project failed once. Then failed the exact same way.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>skipped-the-debrief-repeated-the-failure</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/skipped-the-debrief-repeated-the-failure</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>8</v>
+      </c>
+      <c r="J25" t="n">
+        <v>3</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>They owned 50% of the market. Fear owned 100% of the culture.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>nokia-looked-unbeatable-crumbled</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/nokia-looked-unbeatable-crumbled</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>8</v>
+      </c>
+      <c r="J26" t="n">
+        <v>3</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Apple was 90 days from bankrupt. He fired the entire board.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>jobs-told-apple-board-resign</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/jobs-told-apple-board-resign</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>8</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>They fired 5,300 employees. The CEO built the system.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>wells-fargo-blamed-5300-employees</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wells-fargo-blamed-5300-employees</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>8</v>
+      </c>
+      <c r="J28" t="n">
+        <v>3</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>They studied 180 teams. Talent was not the answer.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>google-asked-what-makes-teams-work</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/google-asked-what-makes-teams-work</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>8</v>
+      </c>
+      <c r="J29" t="n">
+        <v>3</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Every chart was green. The company was losing $17 billion.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>mulally-ford-all-green-losing-billions</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/mulally-ford-all-green-losing-billions</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>8</v>
+      </c>
+      <c r="J30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Revenue hit $100 billion. Almost none of it was real.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>enron-punished-dissent-rewarded-fraud</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/enron-punished-dissent-rewarded-fraud</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9) - YouTube 429</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>8</v>
+      </c>
+      <c r="J31" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1461,13 +1971,13 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>6</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -1482,13 +1992,13 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>6</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -1503,17 +2013,17 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -1524,17 +2034,17 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -1545,17 +2055,17 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>4</v>
-      </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -1566,17 +2076,17 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>4</v>
-      </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -1627,7 +2137,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -1650,7 +2160,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>First batch created 2026-03-24</t>
+          <t>Batch 3 created 2026-03-25. Stories 21-30.</t>
         </is>
       </c>
     </row>
@@ -1665,7 +2175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1780,6 +2290,42 @@
         <v>250</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>21-30</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>dd7cbba</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>89</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1 YouTube 429 (Story 30)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>TikTok/YouTube via customScheduled (daily limits). Pinterest skipped. 4 FICTIONAL + 6 TRUE. Nokia, Apple, Wells Fargo, Google, Ford, Enron.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1791,7 +2337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2080,6 +2626,156 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>25</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Nokia smartphone failure</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>50% market share 2007, fear-based culture, truth-tellers labeled losers, sold to Microsoft 2013, 50% to &lt;3% in 6 years</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>INSEAD, tandfonline, brandminds</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>26</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Apple/Jobs 1997 return</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>90 days from bankruptcy, fired board except Woolard, slashed products 70%, $150M Microsoft deal, 4 product quadrants</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TIME, Macworld, mediashower</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>27</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Wells Fargo fake accounts</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1.5M fake accounts, 500K unauthorized cards, 5300 fired, Stumpf resigned Oct 2016, $3B+ fines, eight is great</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Harvard Law, SEC, Wikipedia</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>28</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Google Project Aristotle</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>180 teams studied 2012, psych safety 43% variance, 19% productivity, 31% innovation, 27% lower turnover</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>psychsafety.com, rework.withgoogle, leaderfactor</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>29</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ford/Mulally turnaround</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Losing $17B 2006, all-green charts, Mark Fields first red slide, Mulally clapped, no bailout needed, weekly BPR</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>chiefexecutive.net, kornferry, medium</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>30</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Enron collapse</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>$13B to $100B in 4 years, mark-to-market, rank and yank, Sherron Watkins memo, $90 to &lt;$1, Skilling 24 years</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>scu.edu, kornferry, fourweekmba</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update story-tracker.xlsx after run #4
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1911,6 +1911,516 @@
         <v>3</v>
       </c>
       <c r="K31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Engagement was at 94%. Nobody was engaged.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>engagement-94-nobody-engaged</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/engagement-94-nobody-engaged</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>8</v>
+      </c>
+      <c r="J32" t="n">
+        <v>3</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>The CEO talked for 55 minutes. Then asked for input.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>ceo-talked-55-minutes</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/ceo-talked-55-minutes</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>8</v>
+      </c>
+      <c r="J33" t="n">
+        <v>3</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Three new hires. Same role. All quit within a year.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>three-hires-same-role-all-quit</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/three-hires-same-role-all-quit</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>8</v>
+      </c>
+      <c r="J34" t="n">
+        <v>3</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>She asked one question. Half the room started crying.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>one-question-half-room-crying</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/one-question-half-room-crying</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>8</v>
+      </c>
+      <c r="J35" t="n">
+        <v>3</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Two departments. Same data. Opposite conclusions.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>same-data-opposite-conclusions</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/same-data-opposite-conclusions</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>8</v>
+      </c>
+      <c r="J36" t="n">
+        <v>3</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>They celebrated the launch. Nobody mentioned the risk.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>celebrated-launch-ignored-risk</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/celebrated-launch-ignored-risk</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>8</v>
+      </c>
+      <c r="J37" t="n">
+        <v>3</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Every manager had a plan. Fire the bottom 10%.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>ge-rank-and-yank-fire-bottom</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/ge-rank-and-yank-fire-bottom</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>8</v>
+      </c>
+      <c r="J38" t="n">
+        <v>3</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Every advisor said strike. The president left the room.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>jfk-excomm-left-the-room</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/jfk-excomm-left-the-room</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>8</v>
+      </c>
+      <c r="J39" t="n">
+        <v>3</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>The engineers said no. Management said launch.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>challenger-engineers-said-no</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/challenger-engineers-said-no</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>8</v>
+      </c>
+      <c r="J40" t="n">
+        <v>3</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Intel was dying. One question saved it.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>grove-intel-one-question-saved</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/grove-intel-one-question-saved</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>8</v>
+      </c>
+      <c r="J41" t="n">
+        <v>3</v>
+      </c>
+      <c r="K41" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1971,17 +2481,17 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1992,17 +2502,17 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -2013,17 +2523,17 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -2034,17 +2544,17 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -2055,17 +2565,17 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>3</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -2076,17 +2586,17 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>3</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -2137,7 +2647,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -2160,7 +2670,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch 3 created 2026-03-25. Stories 21-30.</t>
+          <t>Batch 4 created 2026-03-25. Stories 31-40. 6 FICTIONAL + 4 TRUE.</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2326,6 +2836,42 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>31-40</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>f25aa8a</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>90</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>TikTok/YouTube daily limits (customScheduled), 1 rate limit pause</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>6 FICTIONAL + 4 TRUE. GE rank-yank, JFK ExComm, Challenger, Intel Grove. Pinterest skipped.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2337,7 +2883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2776,6 +3322,106 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>37</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>GE Rank and Yank</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Jack Welch Vitality Curve 1980s. 20-70-10 system. Bottom 10% fired. Revenue doubled but collaboration destroyed. Abandoned 2016.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Medium, Wikipedia, business.com</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>38</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>JFK ExComm Cuban Missile Crisis</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Oct 1962. 14 advisors. JFK left the room. RFK championed blockade. Soviets backed down.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>JFK Library, Time, National Archives</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>39</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>NASA Challenger O-ring failure</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Jan 27 1986. Thiokol engineers warned. Mason told Lund: take off engineering hat. 73 seconds after launch, broke apart. 7 killed.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>NPR, NASA Rogers Report, Wikipedia</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>40</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Andy Grove Intel strategic inflection</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1985. Grove asked Moore: if we got kicked out, what would new CEO do? Exited memory, bet on microprocessors.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>SkillPacks, Medium, Commoncog</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update story-tracker.xlsx after run #5
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2421,6 +2421,516 @@
         <v>3</v>
       </c>
       <c r="K41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Best-selling pizza chain. Worst pizza in America.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>dominos-worst-pizza-turnaround</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/dominos-worst-pizza-turnaround</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9)</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>8</v>
+      </c>
+      <c r="J42" t="n">
+        <v>3</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Great strategy deck. Dead team behind it.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>great-strategy-dead-team</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/great-strategy-dead-team</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9)</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>8</v>
+      </c>
+      <c r="J43" t="n">
+        <v>3</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>They laughed at the pitch. Then went bankrupt.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>blockbuster-laughed-netflix-bankrupt</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/blockbuster-laughed-netflix-bankrupt</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>8</v>
+      </c>
+      <c r="J44" t="n">
+        <v>3</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Saved $2 million. Lost $20 million.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>saved-two-million-lost-twenty</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/saved-two-million-lost-twenty</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>8</v>
+      </c>
+      <c r="J45" t="n">
+        <v>3</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Worth $28 billion. Missing $2 billion.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>wirecard-missing-billions</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wirecard-missing-billions</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9)</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>8</v>
+      </c>
+      <c r="J46" t="n">
+        <v>3</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Zero incidents reported. Nobody felt safe.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>zero-incidents-nobody-safe</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/zero-incidents-nobody-safe</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9)</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>8</v>
+      </c>
+      <c r="J47" t="n">
+        <v>3</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>He banned slides. The thinking got better.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>bezos-banned-slides-better-thinking</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/bezos-banned-slides-better-thinking</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9)</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>8</v>
+      </c>
+      <c r="J48" t="n">
+        <v>3</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>The loudest voice went silent. Everything changed.</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>loudest-voice-went-silent</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/loudest-voice-went-silent</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9)</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>8</v>
+      </c>
+      <c r="J49" t="n">
+        <v>3</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>They blamed the drivers. 124 people died.</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>gm-blamed-drivers-124-died</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/gm-blamed-drivers-124-died</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9)</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>8</v>
+      </c>
+      <c r="J50" t="n">
+        <v>3</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>He talked about safety. Investors ran for the exit.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>oneill-alcoa-safety-investors-ran</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/oneill-alcoa-safety-investors-ran</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9)</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>8</v>
+      </c>
+      <c r="J51" t="n">
+        <v>3</v>
+      </c>
+      <c r="K51" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2481,17 +2991,17 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -2502,17 +3012,17 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -2523,17 +3033,17 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -2544,17 +3054,17 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -2565,13 +3075,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -2586,13 +3096,13 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -2647,7 +3157,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
@@ -2670,7 +3180,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch 4 created 2026-03-25. Stories 31-40. 6 FICTIONAL + 4 TRUE.</t>
+          <t>Batch 5 created 2026-03-25. Stories 41-50. 6 TRUE + 4 FICTIONAL.</t>
         </is>
       </c>
     </row>
@@ -2685,7 +3195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2872,6 +3382,34 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>41-50</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>6 TRUE + 4 FICTIONAL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>81/90 (9 YouTube failed - daily limit)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2883,7 +3421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3422,6 +3960,156 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>41</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Domino's Pizza turnaround</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Dead last in taste survey 2009, Patrick Doyle aired feedback on TV, rebuilt recipe, stock $3 to $400+, 14.3% same-store sales jump year 1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>restaurantbusinessonline, producthabits, businessage</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>43</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Blockbuster rejected Netflix</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2000 meeting in Dallas, $50M offer, John Antioco laughed, dot-com hysteria overblown, Netflix now $400B+, Blockbuster bankrupt 2010</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>fortune, variety, inc.com</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>45</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Wirecard fraud</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1.9B euros missing/never existed, Markus Braun arrested, Jan Marsalek fled to Belarus, Dan McCrum FT journalist investigated by BaFin, $28B valuation to zero</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>wikipedia, bloomberg, eqs.com</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>47</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Amazon six-page memo</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Bezos banned PowerPoint June 2004, 6-page narrative memos, 30min silent reading, 'smartest thing we ever did', forced rigorous thinking</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>cnbc, inc.com, medium</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>49</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>GM ignition switch scandal</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Faulty switch discovered 2001, TSB 2005 told dealers 'remove heavy keychains', 124 deaths, 30M vehicles recalled 2014, Mary Barra fired 15, $2B+ fines</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>wikipedia, npr, fortune</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>50</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Paul O'Neill Alcoa safety</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CEO Oct 1987, 'I want to talk about worker safety', investor sold shares, market value $3B to $27.5B, injuries 1.86 to 0.2 per 100 workers</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>workclout, bbntimes, psychsafety</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update story-tracker.xlsx after run #6 (stories 51-60)
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2931,6 +2931,516 @@
         <v>3</v>
       </c>
       <c r="K51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Four project managers. Same broken project.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>four-pms-same-broken-project</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/four-pms-same-broken-project</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>8</v>
+      </c>
+      <c r="J52" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>She asked who benefits. Silence.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>asked-who-benefits-silence</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asked-who-benefits-silence</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>8</v>
+      </c>
+      <c r="J53" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Nine months of perfection. One wrong unit.</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>mars-orbiter-one-wrong-unit</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/mars-orbiter-one-wrong-unit</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>8</v>
+      </c>
+      <c r="J54" t="n">
+        <v>3</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Offered $44 billion. They said no.</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>yahoo-said-no-to-44-billion</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/yahoo-said-no-to-44-billion</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>8</v>
+      </c>
+      <c r="J55" t="n">
+        <v>3</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Five-star reviews. Five resignations.</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>five-star-reviews-five-resignations</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-star-reviews-five-resignations</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>8</v>
+      </c>
+      <c r="J56" t="n">
+        <v>3</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>The intern spoke. The room froze.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>intern-spoke-room-froze</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/intern-spoke-room-froze</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9)</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>8</v>
+      </c>
+      <c r="J57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Zero injuries recorded. Eleven people died.</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>bp-zero-injuries-eleven-died</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/bp-zero-injuries-eleven-died</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>8</v>
+      </c>
+      <c r="J58" t="n">
+        <v>3</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Right question. Wrong answer. 800,000 customers left.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>netflix-right-question-wrong-answer</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/netflix-right-question-wrong-answer</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>8</v>
+      </c>
+      <c r="J59" t="n">
+        <v>3</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Dashboard was green. Clients were gone.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>dashboard-green-clients-gone</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/dashboard-green-clients-gone</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>8</v>
+      </c>
+      <c r="J60" t="n">
+        <v>3</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>They cut training first. Then wondered why.</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>cut-training-wondered-why</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/cut-training-wondered-why</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>8</v>
+      </c>
+      <c r="J61" t="n">
+        <v>3</v>
+      </c>
+      <c r="K61" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2991,17 +3501,17 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>5</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -3012,17 +3522,17 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>5</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -3033,13 +3543,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -3054,13 +3564,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -3075,13 +3585,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3606,13 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -3157,7 +3667,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
@@ -3180,7 +3690,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch 5 created 2026-03-25. Stories 41-50. 6 TRUE + 4 FICTIONAL.</t>
+          <t>Batch 6 created 2026-03-25. Stories 51-60. 4 TRUE + 6 FICTIONAL.</t>
         </is>
       </c>
     </row>
@@ -3195,7 +3705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3410,6 +3920,42 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>51-60</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>b6130c7a</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>89</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>TikTok/YouTube daily limits (customScheduled), 1 X/Twitter duplicate (Story 56)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>4 TRUE + 6 FICTIONAL. Mars Orbiter, Yahoo/Microsoft, BP Deepwater Horizon, Netflix/Qwikster. Pinterest skipped.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3421,7 +3967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4110,6 +4656,106 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>53</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>NASA Mars Climate Orbiter</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Launched Dec 1998, $327M mission. Lockheed Martin used imperial (pound-force seconds), NASA expected metric (newton-seconds). Lost Sep 23 1999, flew 170km too close. 9 months accumulated error.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Wikipedia, NASA, SimScale, Everyday Astronaut</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>54</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Yahoo rejects Microsoft $44.6B</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Feb 2008, 62% premium. Jerry Yang said 'substantially undervalues'. Refused counter-offer. Stock collapsed. Carl Icahn proxy fight. Yang resigned Nov 2008. Verizon bought for $4.8B in 2016.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>CNBC, Wikipedia, UCLA, Quora</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>57</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>BP Deepwater Horizon</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Personal safety record looked good (helmets, slip-and-fall). Process safety ignored. Apr 20 2010, 11 killed, 4.9M barrels over 87 days. BP blamed workers, U.S. found systemic failures.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Chemistry World, EHS Today, MIT Sloan, CorpWatch</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>58</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Netflix Qwikster pivot</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>24M subs in 2011. Hastings split DVD/streaming into Netflix + Qwikster. 60% price hike. 800K cancelled in Q3 2011. Stock dropped 77%. Killed Qwikster in 3 weeks. 280M subs by 2024.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Medium, MIT Tech Review, NPR, QZ</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update story-tracker.xlsx after run #7
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3441,6 +3441,516 @@
         <v>3</v>
       </c>
       <c r="K61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>She fired the fundraiser. Donations kept falling.</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>fired-fundraiser-donations-falling</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/fired-fundraiser-donations-falling</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>8</v>
+      </c>
+      <c r="J62" t="n">
+        <v>3</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>He asked why. Five times. Everything shifted.</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>asked-why-five-times-shifted</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asked-why-five-times-shifted</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>8</v>
+      </c>
+      <c r="J63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Seven people died. He recalled 31 million bottles.</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>jj-tylenol-recalled-31-million</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/jj-tylenol-recalled-31-million</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>8</v>
+      </c>
+      <c r="J64" t="n">
+        <v>3</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>$529 million in pay. $600 billion in losses.</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>lehman-fuld-529m-600b-losses</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/lehman-fuld-529m-600b-losses</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>8</v>
+      </c>
+      <c r="J65" t="n">
+        <v>3</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Worth $47 billion. Couldn't explain the math.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>wework-47b-couldnt-explain-math</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wework-47b-couldnt-explain-math</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>8</v>
+      </c>
+      <c r="J66" t="n">
+        <v>3</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>He closed 7,100 stores. In one afternoon.</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>schultz-closed-7100-stores</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/schultz-closed-7100-stores</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>8</v>
+      </c>
+      <c r="J67" t="n">
+        <v>3</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>She banned remote work. The problem was deeper.</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>mayer-yahoo-banned-remote-deeper</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/mayer-yahoo-banned-remote-deeper</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>8</v>
+      </c>
+      <c r="J68" t="n">
+        <v>3</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>One question, asked five times. Toyota was born.</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ohno-toyota-five-whys-born</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/ohno-toyota-five-whys-born</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>8</v>
+      </c>
+      <c r="J69" t="n">
+        <v>3</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Perfect hire. Wrong role. She saw it too late.</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>perfect-hire-wrong-role-too-late</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/perfect-hire-wrong-role-too-late</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>8</v>
+      </c>
+      <c r="J70" t="n">
+        <v>3</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>They skipped the hard conversation. Twice.</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>skipped-hard-conversation-twice</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/skipped-hard-conversation-twice</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>8</v>
+      </c>
+      <c r="J71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K71" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3501,17 +4011,17 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>6</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -3522,17 +4032,17 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>6</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -3543,13 +4053,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -3564,13 +4074,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -3585,13 +4095,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -3606,13 +4116,13 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -3667,7 +4177,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4">
@@ -3690,7 +4200,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch 6 created 2026-03-25. Stories 51-60. 4 TRUE + 6 FICTIONAL.</t>
+          <t>Batch 7 created 2026-03-25. Stories 61-70. 6 TRUE + 4 FICTIONAL.</t>
         </is>
       </c>
     </row>
@@ -3705,7 +4215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3956,6 +4466,42 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>61-70</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>10e691de</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>90</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>TikTok/YouTube daily limits (customScheduled), 3 Instagram retries</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>6 TRUE + 4 FICTIONAL. J&amp;J Tylenol, Lehman Brothers, WeWork, Starbucks/Schultz, Yahoo/Mayer, Toyota/Ohno. Pinterest skipped.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3967,7 +4513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4756,6 +5302,96 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>63</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>J&amp;J Tylenol crisis 1982</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>James Burke recalled 31M bottles of Tylenol after 7 cyanide deaths in Chicago. FBI/FDA advised against. Cost $100M. Market share crashed 35% to 7%, recovered within a year. Gold standard crisis management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>64</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Lehman Brothers collapse 2008</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Dick Fuld ignored liquidity warnings, spent $10B on bonuses/buybacks. Filed bankruptcy Sep 15 2008. $600B assets gone. Triggered worst financial crisis since Great Depression. Fuld earned $529M 2000-2007.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>65</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>WeWork IPO failure 2019</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Adam Neumann's WeWork valued at $47B. S-1 revealed 'community-adjusted EBITDA', self-dealing. IPO pulled. Neumann forced out with $1.7B. Filed bankruptcy Nov 2023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>66</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Starbucks Schultz return 2008</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Howard Schultz returned as CEO Jan 2008. Closed all 7,100 US stores Feb 26 for 3 hours to retrain 135,000 employees. Added ~$100B market value 2008-2017.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>67</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Yahoo Marissa Mayer 2012-2016</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Mayer became CEO 2012. Banned remote work Feb 2013. Introduced bell-curve rankings. Treated strategy problem as people problem. Yahoo sold to Verizon for $4.5B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>68</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Toyota Five Whys Taiichi Ohno</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Taiichi Ohno developed Five Whys method in 1950s. Ask 'why' 5 times to find root cause. Became foundation of Toyota Production System. Toyota grew to world's largest automaker.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update story-tracker.xlsx after run #8
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K71"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3951,6 +3951,516 @@
         <v>3</v>
       </c>
       <c r="K71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Retention was 96%. Nobody was staying by choice.</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>retention-96-nobody-staying-by-choice</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/retention-96-nobody-staying-by-choice</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9) - YouTube daily limit</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>8</v>
+      </c>
+      <c r="J72" t="n">
+        <v>3</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>She cancelled the agenda. The truth came out.</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>cancelled-agenda-truth-came-out</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/cancelled-agenda-truth-came-out</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9) - YouTube daily limit</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>8</v>
+      </c>
+      <c r="J73" t="n">
+        <v>3</v>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Three principals. Five years. Same complaints.</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>three-principals-same-complaints</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/three-principals-same-complaints</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9) - YouTube daily limit</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>8</v>
+      </c>
+      <c r="J74" t="n">
+        <v>3</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>He asked what to stop. Nobody could answer.</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>asked-what-to-stop-no-answer</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asked-what-to-stop-no-answer</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9) - YouTube daily limit</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>8</v>
+      </c>
+      <c r="J75" t="n">
+        <v>3</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>The alarm went off. Nobody looked.</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>target-alarm-nobody-looked</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/target-alarm-nobody-looked</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9) - YouTube daily limit</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>8</v>
+      </c>
+      <c r="J76" t="n">
+        <v>3</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>$6 billion in debt. Then they blamed Amazon.</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>toys-r-us-blamed-amazon</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/toys-r-us-blamed-amazon</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9) - YouTube daily limit</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>8</v>
+      </c>
+      <c r="J77" t="n">
+        <v>3</v>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>12,000 stores open. $300 million was fake.</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>luckin-12000-stores-fake</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/luckin-12000-stores-fake</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9) - YouTube daily limit</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>8</v>
+      </c>
+      <c r="J78" t="n">
+        <v>3</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Losing $1 million a day. He called it a burning platform.</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>lego-burning-platform-million-a-day</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/lego-burning-platform-million-a-day</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9) - YouTube daily limit</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>8</v>
+      </c>
+      <c r="J79" t="n">
+        <v>3</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Blamed one developer. 87 million were exposed.</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>facebook-blamed-developer-87m-exposed</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/facebook-blamed-developer-87m-exposed</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9) - YouTube daily limit</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>8</v>
+      </c>
+      <c r="J80" t="n">
+        <v>3</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Better milkshake. Same sales. Wrong question.</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>christensen-milkshake-wrong-question</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/christensen-milkshake-wrong-question</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Scheduled (8/9) - YouTube daily limit</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>8</v>
+      </c>
+      <c r="J81" t="n">
+        <v>3</v>
+      </c>
+      <c r="K81" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4011,17 +4521,17 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -4032,17 +4542,17 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -4053,13 +4563,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -4074,13 +4584,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -4095,17 +4605,17 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>6</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -4116,17 +4626,17 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>6</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -4177,7 +4687,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4">
@@ -4200,7 +4710,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch 7 created 2026-03-25. Stories 61-70. 6 TRUE + 4 FICTIONAL.</t>
+          <t>Batch 8 created 2026-03-26. Stories 71-80. 6 TRUE + 4 FICTIONAL.</t>
         </is>
       </c>
     </row>
@@ -4215,7 +4725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4502,6 +5012,42 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>71-80</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>cfd526c3</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>80</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>YouTube daily limit (10/10 failed), TikTok daily limit (7 via customScheduled)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>4 FICTIONAL + 6 TRUE. Target data breach, Toys R Us/KKR, Luckin Coffee, LEGO/Knudstorp, Facebook/Cambridge Analytica, Christensen JTBD. Pinterest skipped.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4513,7 +5059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5392,6 +5938,156 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>75</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Target data breach 2013</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>FireEye system installed, Bangalore team flagged Nov 30, Minneapolis ignored for 12 days, 40M cards stolen, $200M+ costs, CEO and CIO fired</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>CEI, Slate, Senate Commerce, Medium</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>76</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Toys R Us KKR leveraged buyout</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>KKR/Bain/Vornado 2005 LBO, $6B debt, $500M/yr interest, $2.2B reserves to $301M, profitable without debt, 33K jobs lost, 800 stores closed</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>American Prospect, Columbia Law, MIT Sloan</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>77</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Luckin Coffee fraud 2020</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>4500+ locations, $12B valuation, COO fabricated $300M+ sales, shell companies with fake vouchers, stock fell 97%, delisted after 13 months, $180M SEC penalty</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>SEC, CNBC, HBS, Seven Pillars</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>78</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>LEGO near-bankruptcy Knudstorp</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Losing $1M/day 2003, 13000 SKUs, $800M debt, Knudstorp "burning platform" report, made CEO 2004, cut to 7000 SKUs, sold theme parks, became most valuable toy company</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>BCG, CEO Magazine, Strategy Institute</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>79</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Facebook Cambridge Analytica</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Kogan harvested 87M users via Open Graph API, data to Cambridge Analytica, Facebook banned Kogan but API was designed that way, $120B lost in one day, $5B FTC fine</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Wikipedia, CNBC, Slate, Senate Judiciary</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>80</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Christensen Jobs to Be Done milkshake</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Fast food chain, made shakes better, sales flat, Christensen asked "what job hired to do", morning commuters, competition was bananas/bagels/boredom, sales up 7x</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>HBR, Christensen Institute, Rewired Group, HBS Online</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update story-tracker.xlsx after run #9
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K81"/>
+  <dimension ref="A1:K91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4461,6 +4461,516 @@
         <v>3</v>
       </c>
       <c r="K81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Perfect strategy. Wrong problem.</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>perfect-strategy-wrong-problem</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/perfect-strategy-wrong-problem</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>8</v>
+      </c>
+      <c r="J82" t="n">
+        <v>3</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Promoted the star. Lost the team.</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>promoted-star-lost-team</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/promoted-star-lost-team</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>8</v>
+      </c>
+      <c r="J83" t="n">
+        <v>3</v>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>30 divisions competed. Zero served customers.</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>sears-30-divisions-zero-customers</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/sears-30-divisions-zero-customers</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>8</v>
+      </c>
+      <c r="J84" t="n">
+        <v>3</v>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Laid off 1,900 people. They thanked him.</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>chesky-laid-off-thanked-him</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/chesky-laid-off-thanked-him</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>8</v>
+      </c>
+      <c r="J85" t="n">
+        <v>3</v>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Five teachers quit. Blamed all five.</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>five-teachers-blamed-all-five</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-teachers-blamed-all-five</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>8</v>
+      </c>
+      <c r="J86" t="n">
+        <v>3</v>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Asked why. Nobody had an answer.</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>asked-why-nobody-answered</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asked-why-nobody-answered</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>8</v>
+      </c>
+      <c r="J87" t="n">
+        <v>3</v>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>$3.4B in revenue. A dead end ahead.</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>adobe-billions-dead-end</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/adobe-billions-dead-end</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>8</v>
+      </c>
+      <c r="J88" t="n">
+        <v>3</v>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Called it a toy. It killed his company.</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>blackberry-called-it-toy</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/blackberry-called-it-toy</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>8</v>
+      </c>
+      <c r="J89" t="n">
+        <v>3</v>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Meetings on time. Nothing decided.</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>meetings-on-time-nothing-decided</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/meetings-on-time-nothing-decided</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>8</v>
+      </c>
+      <c r="J90" t="n">
+        <v>3</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Cancelled the meeting. Output doubled.</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>cancelled-meeting-output-doubled</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/cancelled-meeting-output-doubled</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>8</v>
+      </c>
+      <c r="J91" t="n">
+        <v>3</v>
+      </c>
+      <c r="K91" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4521,13 +5031,13 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -4542,13 +5052,13 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -4563,13 +5073,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>8</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -4584,13 +5094,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>8</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -4605,13 +5115,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" s="2" t="n">
         <v>7</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>6</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -4626,13 +5136,13 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C7" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" s="2" t="n">
         <v>7</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>6</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -4687,7 +5197,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4">
@@ -4710,7 +5220,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch 8 created 2026-03-26. Stories 71-80. 6 TRUE + 4 FICTIONAL.</t>
+          <t>Batch 9 created 2026-03-26. Stories 81-90. 4 TRUE + 6 FICTIONAL.</t>
         </is>
       </c>
     </row>
@@ -4725,7 +5235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5048,6 +5558,44 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>81-90</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>b41f3908 (Git Data API)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>90 posts (9 platforms x 10 stories)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>TikTok/YouTube daily limits (switched to customScheduled)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>4 TRUE (Sears, Airbnb/Chesky, Adobe, BlackBerry) + 6 FICTIONAL. GitHub clone failed (disk space), used Git Data API instead. TikTok customScheduled Apr 2-11, YouTube customScheduled Apr 20-29.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5059,7 +5607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6088,6 +6636,106 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>83</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Sears internal division competition</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Sears organized into 30+ business units that competed against each other. Eddie Lampert's strategy led to internal warfare. Divisions refused to cooperate, leading to decline and 2018 bankruptcy.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Bloomberg, WSJ, business case studies</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>84</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Airbnb COVID layoffs by Brian Chesky</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>In May 2020, Chesky laid off 1,900 employees (25% of workforce). His transparent letter praised employees, offered generous severance, extended healthcare, and created an alumni talent directory. Widely praised as model of compassionate leadership.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Chesky open letter May 2020, HBR analysis, NYT coverage</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>87</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Adobe Creative Cloud pivot</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Under Shantanu Narayen, Adobe shifted from boxed software to Creative Cloud subscription model in 2013. Revenue initially dropped but eventually grew from $4B to $17B+. Considered one of the most successful business model pivots in tech.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Adobe annual reports, Forbes, Wired analysis</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>88</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>BlackBerry dismissing iPhone</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>In 2007, BlackBerry co-CEO Jim Balsillie and Mike Lazaridis dismissed the iPhone as 'not a threat' and 'an IT manager's worst nightmare.' By 2016 BlackBerry had effectively exited the smartphone market. Peak market share ~50% dropped to &lt;1%.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Bloomberg retrospectives, The Verge, business case studies</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update story-tracker.xlsx after run #10
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4971,6 +4971,516 @@
         <v>3</v>
       </c>
       <c r="K91" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Replaced half the team. Same results.</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>replaced-half-same-results</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/replaced-half-same-results</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>8</v>
+      </c>
+      <c r="J92" t="n">
+        <v>3</v>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>One question. Twelve silent faces.</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>one-question-twelve-silent</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/one-question-twelve-silent</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>8</v>
+      </c>
+      <c r="J93" t="n">
+        <v>3</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Record fundraising year. Staff in tears.</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>record-year-staff-in-tears</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/record-year-staff-in-tears</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>8</v>
+      </c>
+      <c r="J94" t="n">
+        <v>3</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Saved $2M. Lost every senior leader.</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>saved-2m-lost-senior-leaders</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/saved-2m-lost-senior-leaders</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>8</v>
+      </c>
+      <c r="J95" t="n">
+        <v>3</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Invented the future. Let others sell it.</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>xerox-invented-future-others-sold</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/xerox-invented-future-others-sold</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>8</v>
+      </c>
+      <c r="J96" t="n">
+        <v>3</v>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Called it a crazy idea. It saved Disney.</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>iger-crazy-idea-saved-disney</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/iger-crazy-idea-saved-disney</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>8</v>
+      </c>
+      <c r="J97" t="n">
+        <v>3</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Ranked every employee. Lost the best ones.</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>microsoft-ranked-lost-best</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/microsoft-ranked-lost-best</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>8</v>
+      </c>
+      <c r="J98" t="n">
+        <v>3</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Laid off a third. The rest got better.</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>netflix-laid-off-third-got-better</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/netflix-laid-off-third-got-better</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>8</v>
+      </c>
+      <c r="J99" t="n">
+        <v>3</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Everyone wrote it off. He walked the floor.</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>bestbuy-joly-walked-floor</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/bestbuy-joly-walked-floor</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>8</v>
+      </c>
+      <c r="J100" t="n">
+        <v>3</v>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Stock up 600%. Then it all collapsed.</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>peloton-600-percent-collapsed</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/peloton-600-percent-collapsed</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>8</v>
+      </c>
+      <c r="J101" t="n">
+        <v>3</v>
+      </c>
+      <c r="K101" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5031,17 +5541,17 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -5052,17 +5562,17 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>8</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -5073,13 +5583,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -5094,13 +5604,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -5115,13 +5625,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -5136,13 +5646,13 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -5197,7 +5707,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>91</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4">
@@ -5220,7 +5730,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch 9 created 2026-03-26. Stories 81-90. 4 TRUE + 6 FICTIONAL.</t>
+          <t>Batch 10 created 2026-03-26. Stories 91-100. 4 FICTIONAL + 6 TRUE.</t>
         </is>
       </c>
     </row>
@@ -5235,7 +5745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5596,6 +6106,44 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>91-100</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>44181924 (Git Data API)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>90 posts (9 platforms x 10 stories)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>TikTok/YouTube daily limits (switched to customScheduled). TikTok Apr 12-21, YouTube Apr 30 - May 9.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>4 FICTIONAL + 6 TRUE. Xerox PARC, Disney/Iger Pixar, Microsoft stack ranking, Netflix keeper test, Best Buy/Joly, Peloton/Foley. Pinterest skipped (no boards). Story 100 milestone!</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5607,7 +6155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6736,6 +7284,156 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>95</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Xerox PARC GUI invention</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Xerox PARC invented GUI, mouse, Ethernet in 1970s. Steve Jobs visited Dec 1979. Xerox Star 1981 at $16,595 failed commercially. Apple/Microsoft built on PARC ideas.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Stanford, Wikipedia, Mac History</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>96</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Disney Pixar acquisition Bob Iger</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Iger called Jobs late 2005 with 'crazy idea.' Pixar acquired for $7.4B in 2006. Jobs became Disney's largest shareholder. Led to Frozen, Tangled, Moana.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>CNBC, TheWrap, MasterClass</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>97</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Microsoft Ballmer stack ranking</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Stack ranking under Ballmer forced bell curve rankings. Every employee Eichenwald interviewed cited it as most destructive process. Abandoned 2013. Nadella replaced with growth mindset. Stock $38 to $400+.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Slate, Ricky Spears, NPR</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>98</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Netflix keeper test origin</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Dot-com bust 2001, Netflix laid off a third. Remaining team accelerated. Hastings asked 'Would I fight to keep this person?' Became 125-page culture deck viewed 5M+ times.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Netflix Jobs, Substack, Quartz</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>99</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Best Buy Hubert Joly turnaround</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Joly hired 2012 as hospitality exec. Spent first week on store floor in St. Cloud MN. Launched Renew Blue. 335% total shareholder return vs 104% S&amp;P 500 over 7 years.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>McKinsey, Best Buy Corporate, StarTribune</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>100</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Peloton John Foley overexpansion</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Pandemic: stock up 600%. Foley expanded aggressively. Gyms reopened, demand collapsed. Stock dropped 75%. Feb 2022: 2,800 laid off, Foley stepped down. $800M restructuring.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>NPR, WashPost, TechCrunch, Fortune</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update story-tracker.xlsx after run #11
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5481,6 +5481,516 @@
         <v>3</v>
       </c>
       <c r="K101" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Perfect attendance. Nobody present.</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>perfect-attendance-nobody-present</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/perfect-attendance-nobody-present</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>8</v>
+      </c>
+      <c r="J102" t="n">
+        <v>3</v>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Asked for the truth. One person spoke.</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>asked-for-truth-one-spoke</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asked-for-truth-one-spoke</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>8</v>
+      </c>
+      <c r="J103" t="n">
+        <v>3</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Changed the culture. The team stayed.</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>changed-team-culture-stayed</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/changed-team-culture-stayed</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>8</v>
+      </c>
+      <c r="J104" t="n">
+        <v>3</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Asked what success looks like. Nobody agreed.</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>asked-success-nobody-agreed</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asked-success-nobody-agreed</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>8</v>
+      </c>
+      <c r="J105" t="n">
+        <v>3</v>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Every department was busy. Nothing connected.</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>every-department-busy-nothing-connected</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/every-department-busy-nothing-connected</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>8</v>
+      </c>
+      <c r="J106" t="n">
+        <v>3</v>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Grew revenue 40%. Lost the mission.</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>grew-revenue-lost-mission</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/grew-revenue-lost-mission</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>8</v>
+      </c>
+      <c r="J107" t="n">
+        <v>3</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Spotify had the perfect structure. Nobody followed it.</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>spotify-perfect-structure-nobody-followed</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/spotify-perfect-structure-nobody-followed</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>8</v>
+      </c>
+      <c r="J108" t="n">
+        <v>3</v>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>A room full of gladiators. He asked for help.</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>nadella-gladiators-asked-for-help</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/nadella-gladiators-asked-for-help</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>8</v>
+      </c>
+      <c r="J109" t="n">
+        <v>3</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Zappos blamed the managers. 18% walked out.</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>zappos-blamed-managers-18-walked-out</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/zappos-blamed-managers-18-walked-out</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>8</v>
+      </c>
+      <c r="J110" t="n">
+        <v>3</v>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Worth $3 billion. He gave it all away.</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>chouinard-patagonia-gave-it-away</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/chouinard-patagonia-gave-it-away</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>8</v>
+      </c>
+      <c r="J111" t="n">
+        <v>3</v>
+      </c>
+      <c r="K111" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5541,17 +6051,17 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>8</v>
-      </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -5562,17 +6072,17 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>8</v>
-      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -5583,17 +6093,17 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C4" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>8</v>
-      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -5604,17 +6114,17 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>9</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -5625,17 +6135,17 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>9</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -5646,17 +6156,17 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C7" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D7" s="2" t="n">
-        <v>8</v>
-      </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -5707,7 +6217,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4">
@@ -5730,7 +6240,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch 10 created 2026-03-26. Stories 91-100. 4 FICTIONAL + 6 TRUE.</t>
+          <t>Batch 11 created 2026-03-26. Stories 101-110. 6 FICTIONAL + 4 TRUE.</t>
         </is>
       </c>
     </row>
@@ -5745,7 +6255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6144,6 +6654,44 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>101-110</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Git Data API batch push (tree 2133463b)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>90 posts (9 platforms x 10 stories)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Buffer 429 on Story 109 YouTube (retried OK). TikTok/YouTube daily limits (switched to customScheduled). TikTok Apr 22-May 1, YouTube May 10-May 19.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>6 FICTIONAL + 4 TRUE. Spotify squad model, Nadella/Microsoft culture, Zappos Holacracy, Chouinard/Patagonia. Pinterest skipped (no boards). Context compaction mid-run (Story 110 scheduling resumed after).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6155,7 +6703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7434,6 +7982,106 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>107</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Spotify Squad Model</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Spotify introduced squad/tribe/chapter/guild model ~2012. Henrik Kniberg documented it. By 2020 many squads had reverted to traditional reporting. Autonomy without alignment created silos. Tribes competed for resources.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Multiple tech sources, Kniberg white paper</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>108</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Nadella Microsoft Culture Shift</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Satya Nadella became Microsoft CEO Jan 2014. Inherited stack-ranking, siloed 'gladiator' culture. Asked leadership team for help openly. Shifted from know-it-all to learn-it-all. Market cap grew from $300B to $3T+.</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Microsoft annual reports, Nadella 'Hit Refresh' book, tech press</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>109</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Zappos Holacracy Experiment</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Tony Hsieh introduced Holacracy at Zappos in 2013-2014. Eliminated traditional managers. Offered buyout to resisters. 18% of workforce (210 people) took the buyout. Company struggled with execution speed.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Multiple business press sources, Zappos internal memos</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>110</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Chouinard Patagonia Ownership Transfer</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Yvon Chouinard transferred Patagonia ownership Sept 2022. Company valued ~$3B. Transferred to Holdfast Collective (nonprofit) and Patagonia Purpose Trust. 'Earth is now our only shareholder.' All profits ($100M/yr) go to climate.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Patagonia press release, NY Times, business press</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update story-tracker.xlsx after run #12
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K111"/>
+  <dimension ref="A1:K121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5991,6 +5991,516 @@
         <v>3</v>
       </c>
       <c r="K111" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>She asked what's right. Wall Street said stop.</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>nooyi-asked-whats-right</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/nooyi-asked-whats-right</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>8</v>
+      </c>
+      <c r="J112" t="n">
+        <v>3</v>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Best soldiers alive. Losing to amateurs.</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>mcchrystal-best-soldiers-losing</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/mcchrystal-best-soldiers-losing</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>8</v>
+      </c>
+      <c r="J113" t="n">
+        <v>3</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Worth $32 billion. None of it was real.</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>ftx-32-billion-none-real</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/ftx-32-billion-none-real</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>8</v>
+      </c>
+      <c r="J114" t="n">
+        <v>3</v>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Day one. He moved to the factory floor.</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>marchionne-day-one-factory-floor</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/marchionne-day-one-factory-floor</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>8</v>
+      </c>
+      <c r="J115" t="n">
+        <v>3</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>They blamed the passenger. The world watched.</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>united-blamed-passenger-world-watched</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/united-blamed-passenger-world-watched</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>8</v>
+      </c>
+      <c r="J116" t="n">
+        <v>3</v>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Raised \$1.75 billion. Dead in six months.</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>quibi-raised-billions-dead-months</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/quibi-raised-billions-dead-months</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>8</v>
+      </c>
+      <c r="J117" t="n">
+        <v>3</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>She asked who we serve. Nobody knew.</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>asked-who-we-serve-nobody-knew</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asked-who-we-serve-nobody-knew</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>8</v>
+      </c>
+      <c r="J118" t="n">
+        <v>3</v>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>The data was perfect. The story was wrong.</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>data-perfect-story-wrong</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/data-perfect-story-wrong</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>8</v>
+      </c>
+      <c r="J119" t="n">
+        <v>3</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Award-winning team. Nobody talked to each other.</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>award-winning-nobody-talked</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/award-winning-nobody-talked</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>8</v>
+      </c>
+      <c r="J120" t="n">
+        <v>3</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>He started with a confession. Everything shifted.</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>started-confession-everything-shifted</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/started-confession-everything-shifted</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>8</v>
+      </c>
+      <c r="J121" t="n">
+        <v>3</v>
+      </c>
+      <c r="K121" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -6051,10 +6561,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>9</v>
@@ -6072,10 +6582,10 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>9</v>
@@ -6093,17 +6603,17 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>9</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -6114,13 +6624,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -6135,13 +6645,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -6156,17 +6666,17 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>9</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -6217,7 +6727,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>111</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4">
@@ -6240,7 +6750,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch 11 created 2026-03-26. Stories 101-110. 6 FICTIONAL + 4 TRUE.</t>
+          <t>Batch 12 created 2026-03-27. Stories 111-120. 6 TRUE + 4 FICTIONAL.</t>
         </is>
       </c>
     </row>
@@ -6255,7 +6765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6692,6 +7202,44 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>111-120</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2f486dfa6</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>90 posts (9 platforms x 10 stories)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>TikTok/YouTube daily limits (customScheduled). Buffer 429 rate limits (recovered). Pinterest skipped.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>6 TRUE (Nooyi/PepsiCo, McChrystal/JSOC, FTX, Marchionne/Chrysler, United Airlines, Quibi) + 4 FICTIONAL. TikTok May 2-11, YouTube May 20-28.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6703,7 +7251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8082,6 +8630,156 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>111</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Indra Nooyi PepsiCo</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>CEO 2006, Performance with Purpose, $2.7B to $6.5B profit, Nelson Peltz pressure, 12yr tenure</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>wartimeceostories, BCG, Duke Fuqua</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>112</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>McChrystal JSOC Team of Teams</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>JSOC 2003-2008, 4 to 300 raids/month, 80/20 flip, shared consciousness, empowered execution</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>foreignpolicy, controlglobal</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>113</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>FTX Sam Bankman-Fried</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>$32B valuation, no audits, $9B missing, CoinDesk Nov 2, bankrupt Nov 11, 25yr prison</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Wikipedia, MIT Sloan, SEC</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>114</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Marchionne Chrysler turnaround</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Fiat 20% June 2009, moved CEO office day 1, 15 reports, profitable &lt;2yr, 16 products 2011</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Fortune, tutor2u, NPR</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>115</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>United Airlines Dr. Dao 2017</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Flight 3411, dragged, Munoz re-accommodating, $1.4B stock drop, policy changes</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Wikipedia, NBC, CNBC, TIME</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>116</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Quibi Katzenberg failure</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>$1.75B raised, 500K vs 7M subs, shut down Oct 2020, Meg Whitman CEO</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Variety, CNBC, Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update batch size to 4 per user request
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -6717,7 +6717,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -6750,7 +6750,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch 12 created 2026-03-27. Stories 111-120. 6 TRUE + 4 FICTIONAL.</t>
+          <t>Batch size changed from 10 to 4 per user request. Batch 12 created 2026-03-27. Stories 111-120. 6 TRUE + 4 FICTIONAL.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update story-tracker.xlsx after run #13
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K121"/>
+  <dimension ref="A1:K125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6504,6 +6504,202 @@
         <is>
           <t>Yes</t>
         </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>The Team That Looks Fine But Isn't</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Sound financial condition. Dead in 48 hours.</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>svb-sound-dead-48-hours</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/svb-sound-dead-48-hours</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>8</v>
+      </c>
+      <c r="J122" t="n">
+        <v>3</v>
+      </c>
+      <c r="K122" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>The Meeting That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Day one as CEO. He killed quarterly reports.</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>polman-killed-quarterly-reports</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/polman-killed-quarterly-reports</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>8</v>
+      </c>
+      <c r="J123" t="n">
+        <v>3</v>
+      </c>
+      <c r="K123" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>The Leader Who Thought It Was a People Problem</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Blamed six teachers. The timetable was broken.</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>blamed-teachers-timetable-broken</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/blamed-teachers-timetable-broken</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>8</v>
+      </c>
+      <c r="J124" t="n">
+        <v>3</v>
+      </c>
+      <c r="K124" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>The Question That Changed Everything</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Membership was dying. One question saved it.</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>hesselbein-girl-scouts-one-question</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/hesselbein-girl-scouts-one-question</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>8</v>
+      </c>
+      <c r="J125" t="n">
+        <v>3</v>
+      </c>
+      <c r="K125" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -6561,17 +6757,17 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>9</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -6582,17 +6778,17 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>9</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -6603,17 +6799,17 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>11</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -6624,17 +6820,17 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FICTIONAL</t>
         </is>
       </c>
     </row>
@@ -6727,7 +6923,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4">
@@ -6750,7 +6946,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch size changed from 10 to 4 per user request. Batch 12 created 2026-03-27. Stories 111-120. 6 TRUE + 4 FICTIONAL.</t>
+          <t>Batch size changed from 10 to 4 per user request. Batch 13 created 2026-03-27. Stories 121-124. 3 TRUE + 1 FICTIONAL.</t>
         </is>
       </c>
     </row>
@@ -6765,7 +6961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7240,6 +7436,44 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>121-124</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>b3463b79</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>36 posts (9 platforms x 4 stories)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>TikTok/YouTube daily limits (customScheduled). 1 Facebook Bad Gateway retry (recovered). 1 X/Twitter 280-char retry (recovered). Pinterest skipped.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>3 TRUE (SVB collapse, Polman/Unilever, Hesselbein/Girl Scouts) + 1 FICTIONAL (school timetable). TikTok May 12-15, YouTube May 29 - Jun 1. Pinterest skipped (no boards).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7251,7 +7485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8780,6 +9014,81 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>121</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SVB collapse 2023</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>16th largest US bank, $209B assets, CRO left Apr 2022, no replacement 8 months, $1.8B loss disclosed Mar 8, $42B withdrawn in one day, seized Mar 10, Fed called it textbook mismanagement</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Wikipedia, Federal Reserve, PYMNTS</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>122</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Paul Polman Unilever</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Became CEO Jan 1 2009, abolished quarterly earnings guidance on day one, stock dropped 8%, launched Sustainable Living Plan, 290% total shareholder return over decade</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Wikipedia, HBR, Fortune, Wartime CEO</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>124</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Frances Hesselbein Girl Scouts</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>CEO 1976-1990, called Peter Drucker pro bono, asked 'What is our mission?', rebuilt around 'help each girl reach her highest potential', membership surged, diversity tripled, Drucker called her best CEO in America</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Jim Collins, Wikipedia, Indiana University</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update story-tracker.xlsx after run #14
</commit_message>
<xml_diff>
--- a/data/carousel-factory/story-tracker.xlsx
+++ b/data/carousel-factory/story-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K125"/>
+  <dimension ref="A1:K129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6699,6 +6699,202 @@
         <v>3</v>
       </c>
       <c r="K125" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Sold guns for 40 years. Then he cried.</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>stack-dicks-sold-guns-then-cried</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/master/carousels/stack-dicks-sold-guns-then-cried</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>8</v>
+      </c>
+      <c r="J126" t="n">
+        <v>3</v>
+      </c>
+      <c r="K126" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>One email destroyed three years of trust.</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>one-email-destroyed-trust</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/master/carousels/one-email-destroyed-trust</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>8</v>
+      </c>
+      <c r="J127" t="n">
+        <v>3</v>
+      </c>
+      <c r="K127" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>The Moment They Saw It</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>FICTIONAL</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Perfect strategy deck. Wrong room entirely.</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>perfect-strategy-wrong-room</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/master/carousels/perfect-strategy-wrong-room</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>8</v>
+      </c>
+      <c r="J128" t="n">
+        <v>3</v>
+      </c>
+      <c r="K128" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>The Cost of Getting It Wrong</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>America's top beer. One post ended it.</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>bud-light-one-post-ended-it</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/master/carousels/bud-light-one-post-ended-it</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Scheduled (9/9)</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>8</v>
+      </c>
+      <c r="J129" t="n">
+        <v>3</v>
+      </c>
+      <c r="K129" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6841,13 +7037,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -6862,17 +7058,17 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>FICTIONAL</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -6923,7 +7119,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4">
@@ -6946,7 +7142,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Batch size changed from 10 to 4 per user request. Batch 13 created 2026-03-27. Stories 121-124. 3 TRUE + 1 FICTIONAL.</t>
+          <t>Batch 14 created 2026-03-27. Stories 125-128. 2 TRUE + 2 FICTIONAL.</t>
         </is>
       </c>
     </row>
@@ -6961,7 +7157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7474,6 +7670,44 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>125-128</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>60fe5a9</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>36 posts (9 platforms x 4 stories)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>TikTok/YouTube daily limits (customScheduled). Pinterest skipped.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2 TRUE (Ed Stack/Dick's, Bud Light/AB InBev) + 2 FICTIONAL (nonprofit email, strategy deck). TikTok May 16-19, YouTube Jun 3-6.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7485,7 +7719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9089,6 +9323,56 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>125</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Ed Stack Dick's Sporting Goods Parkland</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Ed Stack CEO Dick's (850 stores, $9B). After Parkland Feb 2018, pulled all assault-style rifles, raised age to 21, destroyed $5M inventory. $250M+ cost. Gun manufacturers cut ties.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>NPR, CNN, CNBC, Inc, HBR</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>128</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Bud Light AB InBev Dylan Mulvaney 2023</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>April 2023: personalized can to influencer. Conservative boycott. Sales dropped 26%. CEO: 'one post, not a campaign.' Two execs on leave. Lost #1 to Modelo. $1.4B revenue loss, $27B shareholder value lost.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Wikipedia, CNN, The Hill, CBS News</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>